<commit_message>
i think model is finished
</commit_message>
<xml_diff>
--- a/Abschlussprojekt/ProjektLastgang.xlsx
+++ b/Abschlussprojekt/ProjektLastgang.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27932"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10412"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\becker\Documents\HWR\OR\OR 2026\Abschlussprojekt\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/antonia/Documents/01 Uni /01 HWR/05 OR/Abschlussprojekt/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{534A4F6E-E5AE-483E-A568-F6074AF51A3C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{031CBE5C-45C9-0C49-A615-300D0C145FC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-34400" yWindow="-19420" windowWidth="34400" windowHeight="28200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -20,15 +20,12 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="43">
   <si>
     <t>Stunde</t>
   </si>
@@ -127,6 +124,36 @@
   </si>
   <si>
     <t>Sonntags</t>
+  </si>
+  <si>
+    <t>Anlasskosten</t>
+  </si>
+  <si>
+    <t>Anzahl verfügbarer Generatoren</t>
+  </si>
+  <si>
+    <t>Kosten auf Minimallast pro Stunde</t>
+  </si>
+  <si>
+    <t>Kosten oberhalb der Minimallast pro MW und Stunde</t>
+  </si>
+  <si>
+    <t>Minimallast in MW</t>
+  </si>
+  <si>
+    <t>Maximallast in MW</t>
+  </si>
+  <si>
+    <t>Generator 1</t>
+  </si>
+  <si>
+    <t>Generator 2</t>
+  </si>
+  <si>
+    <t>Oberer Puffer</t>
+  </si>
+  <si>
+    <t>Unterer Puffer</t>
   </si>
 </sst>
 </file>
@@ -150,12 +177,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="5">
@@ -222,7 +255,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -239,6 +272,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -519,18 +553,36 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H26"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:AA26"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.1640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="5" max="5" width="12" customWidth="1"/>
+    <col min="1" max="1" width="10.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.5" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="7" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="8" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11.83203125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="10.83203125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="10.1640625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="27.5" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="10.1640625" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="42.1640625" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="10.1640625" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="15.5" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="10.1640625" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="15.6640625" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="10.1640625" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="25.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:27" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:27" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -555,8 +607,32 @@
       <c r="H2" s="2" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="3" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K2" s="6"/>
+      <c r="L2" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="N2" s="6"/>
+      <c r="O2" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q2" s="6"/>
+      <c r="R2" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="T2" s="6"/>
+      <c r="U2" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="W2" s="6"/>
+      <c r="X2" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="Z2" s="6"/>
+      <c r="AA2" s="6" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="3" spans="1:27" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>1</v>
       </c>
@@ -581,8 +657,44 @@
       <c r="H3" s="4">
         <v>1910</v>
       </c>
-    </row>
-    <row r="4" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K3" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="L3">
+        <v>2200</v>
+      </c>
+      <c r="N3" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="O3">
+        <v>600</v>
+      </c>
+      <c r="Q3" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="R3">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="T3" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="U3">
+        <v>500</v>
+      </c>
+      <c r="W3" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="X3">
+        <v>2000</v>
+      </c>
+      <c r="Z3" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="AA3">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="4" spans="1:27" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
@@ -607,8 +719,44 @@
       <c r="H4" s="4">
         <v>1310</v>
       </c>
-    </row>
-    <row r="5" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K4" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="L4">
+        <v>1500</v>
+      </c>
+      <c r="N4" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="O4">
+        <v>900</v>
+      </c>
+      <c r="Q4" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="R4">
+        <v>3.2</v>
+      </c>
+      <c r="T4" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="U4">
+        <v>1500</v>
+      </c>
+      <c r="W4" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="X4">
+        <v>4000</v>
+      </c>
+      <c r="Z4" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="AA4">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5" spans="1:27" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
         <v>3</v>
       </c>
@@ -634,7 +782,7 @@
         <v>1020</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:27" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
         <v>4</v>
       </c>
@@ -660,7 +808,7 @@
         <v>1310</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:27" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
         <v>5</v>
       </c>
@@ -686,7 +834,7 @@
         <v>1480</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:27" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
         <v>6</v>
       </c>
@@ -712,7 +860,7 @@
         <v>1870</v>
       </c>
     </row>
-    <row r="9" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:27" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
         <v>7</v>
       </c>
@@ -738,7 +886,7 @@
         <v>3130</v>
       </c>
     </row>
-    <row r="10" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:27" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>8</v>
       </c>
@@ -764,7 +912,7 @@
         <v>4630</v>
       </c>
     </row>
-    <row r="11" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:27" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
         <v>9</v>
       </c>
@@ -790,7 +938,7 @@
         <v>5310</v>
       </c>
     </row>
-    <row r="12" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:27" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>10</v>
       </c>
@@ -816,7 +964,7 @@
         <v>5920</v>
       </c>
     </row>
-    <row r="13" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:27" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>11</v>
       </c>
@@ -842,7 +990,7 @@
         <v>5950</v>
       </c>
     </row>
-    <row r="14" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:27" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>12</v>
       </c>
@@ -867,8 +1015,14 @@
       <c r="H14" s="4">
         <v>6230</v>
       </c>
-    </row>
-    <row r="15" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K14" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="L14">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="15" spans="1:27" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
         <v>13</v>
       </c>
@@ -893,8 +1047,14 @@
       <c r="H15" s="4">
         <v>7540</v>
       </c>
-    </row>
-    <row r="16" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K15" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="L15">
+        <v>0.15</v>
+      </c>
+    </row>
+    <row r="16" spans="1:27" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>14</v>
       </c>
@@ -920,7 +1080,7 @@
         <v>7320</v>
       </c>
     </row>
-    <row r="17" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:8" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
         <v>15</v>
       </c>
@@ -946,7 +1106,7 @@
         <v>5940</v>
       </c>
     </row>
-    <row r="18" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:8" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
         <v>16</v>
       </c>
@@ -972,7 +1132,7 @@
         <v>5680</v>
       </c>
     </row>
-    <row r="19" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:8" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
         <v>17</v>
       </c>
@@ -998,7 +1158,7 @@
         <v>5560</v>
       </c>
     </row>
-    <row r="20" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:8" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
         <v>18</v>
       </c>
@@ -1024,7 +1184,7 @@
         <v>5370</v>
       </c>
     </row>
-    <row r="21" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:8" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
         <v>19</v>
       </c>
@@ -1050,7 +1210,7 @@
         <v>5220</v>
       </c>
     </row>
-    <row r="22" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:8" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
         <v>20</v>
       </c>
@@ -1076,7 +1236,7 @@
         <v>4580</v>
       </c>
     </row>
-    <row r="23" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:8" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A23" s="3" t="s">
         <v>21</v>
       </c>
@@ -1102,7 +1262,7 @@
         <v>4260</v>
       </c>
     </row>
-    <row r="24" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:8" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A24" s="3" t="s">
         <v>22</v>
       </c>
@@ -1128,7 +1288,7 @@
         <v>4160</v>
       </c>
     </row>
-    <row r="25" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:8" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A25" s="3" t="s">
         <v>23</v>
       </c>
@@ -1154,7 +1314,7 @@
         <v>3070</v>
       </c>
     </row>
-    <row r="26" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:8" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A26" s="3" t="s">
         <v>24</v>
       </c>

</xml_diff>